<commit_message>
fix: corregir IDs de condiciones EST001-EST012 en admin.html y agregar columna Tipo + EST012 Envenenado a la planilla de tienda
</commit_message>
<xml_diff>
--- a/vistas/panel-del-director/Plantilla_Tienda_CDC.xlsx
+++ b/vistas/panel-del-director/Plantilla_Tienda_CDC.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:R7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -491,14 +491,15 @@
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="40" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="40" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -549,40 +550,45 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Equipable</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Ranura</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Contenedor</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Bono</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Estado Asociado</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Quita Condición</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Disponibilidad</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
@@ -628,38 +634,43 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
+          <t>Consumible</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L2" s="2" t="n">
+      <c r="M2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>No Aplica</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>No Aplica</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>No Aplica</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>Común</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>Hidratación básica para el cazador.</t>
         </is>
@@ -705,38 +716,43 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
+          <t>Consumible</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L3" s="2" t="n">
+      <c r="M3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>No Aplica</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>No Aplica</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>EST001</t>
         </is>
       </c>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="Q3" s="2" t="inlineStr">
         <is>
           <t>Común</t>
         </is>
       </c>
-      <c r="Q3" s="2" t="inlineStr">
+      <c r="R3" s="2" t="inlineStr">
         <is>
           <t>Venda básica. Al usarse quita el estado Sangrado.</t>
         </is>
@@ -782,38 +798,43 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
+          <t>Arma</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Mano Derecha o Izquierda</t>
         </is>
       </c>
-      <c r="L4" s="2" t="n">
+      <c r="M4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>+1 Armas Cuerpo a Cuerpo</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>EST001</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>No Aplica</t>
         </is>
       </c>
-      <c r="P4" s="2" t="inlineStr">
+      <c r="Q4" s="2" t="inlineStr">
         <is>
           <t>Escasa</t>
         </is>
       </c>
-      <c r="Q4" s="2" t="inlineStr">
+      <c r="R4" s="2" t="inlineStr">
         <is>
           <t>Hoja robusta para caza. Aplica Sangrado con 3+ éxitos.</t>
         </is>
@@ -859,125 +880,217 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
+          <t>Objeto</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Espalda</t>
         </is>
       </c>
-      <c r="L5" s="2" t="n">
+      <c r="M5" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>No Aplica</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>No Aplica</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>No Aplica</t>
         </is>
       </c>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="Q5" s="2" t="inlineStr">
         <is>
           <t>Escasa</t>
         </is>
       </c>
-      <c r="Q5" s="2" t="inlineStr">
+      <c r="R5" s="2" t="inlineStr">
         <is>
           <t>Mochila resistente para expediciones largas.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="6" ht="35" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>ARM002</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Chaleco de Cuero</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Armadura Ligera</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Torso</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Profesional</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Armadura</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Torso</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>+1 Defensa</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>No Aplica</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>No Aplica</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>Escasa</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>Chaleco reforzado de cuero curtido. Protección ligera sin sacrificar movilidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Ej: BZ001</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Nombre del item</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Alimentación / Arma CaC / Médico / Contenedor...</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Subcategoría o 'No Aplica'</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Común / Profesional / Reforzada / Especializada / Obra de Arte / Única</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Solo número sin $</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Cantidad disponible</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>En kg. Ej: 0.5</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Slots que ocupa en inventario</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>Sí / No</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>Cabeza / Torso / Manos / Piernas / Pies / Cintura / Espalda / Ninguna</t>
-        </is>
-      </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Objeto / Consumible / Arma / Armadura — define si puede ir en una ranura</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>Sí / No — si Tipo es Consumible u Objeto sin Contenedor, debe ser No</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>Ranura o 'Ninguna' — si Tipo es Consumible u Objeto sin Contenedor, debe ser Ninguna</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
         <is>
           <t>Slots que otorga (0 si no es contenedor)</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>+1 Resistencia o 'No Aplica'</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
+      <c r="O7" s="3" t="inlineStr">
         <is>
           <t>EST001 a EST011 o 'No Aplica'</t>
         </is>
       </c>
-      <c r="O6" s="3" t="inlineStr">
+      <c r="P7" s="3" t="inlineStr">
         <is>
           <t>EST001 a EST011 o 'No Aplica'</t>
         </is>
       </c>
-      <c r="P6" s="3" t="inlineStr">
+      <c r="Q7" s="3" t="inlineStr">
         <is>
           <t>Común / Escasa / Rara / Muy Rara / Única</t>
         </is>
       </c>
-      <c r="Q6" s="3" t="inlineStr">
+      <c r="R7" s="3" t="inlineStr">
         <is>
           <t>Descripción narrativa del item</t>
         </is>
@@ -1108,7 +1221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1259,6 +1372,18 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>EST012</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Envenenado</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: columna Acepta para restricción de contenedores, Subcategoría real en municiones, ofertas de armería; admin.html con campos Subcategoría/Acepta/ID/Stock/Disponibilidad/Estado Asociado
</commit_message>
<xml_diff>
--- a/vistas/panel-del-director/Plantilla_Tienda_CDC.xlsx
+++ b/vistas/panel-del-director/Plantilla_Tienda_CDC.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:S7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -493,13 +493,14 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
     <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="40" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="40" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -570,25 +571,30 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>Acepta</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>Bono</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Estado Asociado</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Quita Condición</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Disponibilidad</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
@@ -667,10 +673,15 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
+          <t>No Aplica</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
           <t>Común</t>
         </is>
       </c>
-      <c r="R2" s="2" t="inlineStr">
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>Hidratación básica para el cazador.</t>
         </is>
@@ -744,15 +755,20 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
+          <t>No Aplica</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
           <t>EST001</t>
         </is>
       </c>
-      <c r="Q3" s="2" t="inlineStr">
+      <c r="R3" s="2" t="inlineStr">
         <is>
           <t>Común</t>
         </is>
       </c>
-      <c r="R3" s="2" t="inlineStr">
+      <c r="S3" s="2" t="inlineStr">
         <is>
           <t>Venda básica. Al usarse quita el estado Sangrado.</t>
         </is>
@@ -808,7 +824,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Mano Derecha o Izquierda</t>
+          <t>Mano Der/Izq</t>
         </is>
       </c>
       <c r="M4" s="2" t="n">
@@ -816,25 +832,30 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
+          <t>No Aplica</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
           <t>+1 Armas Cuerpo a Cuerpo</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>EST001</t>
         </is>
       </c>
-      <c r="P4" s="2" t="inlineStr">
-        <is>
-          <t>No Aplica</t>
-        </is>
-      </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
+          <t>No Aplica</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
           <t>Escasa</t>
         </is>
       </c>
-      <c r="R4" s="2" t="inlineStr">
+      <c r="S4" s="2" t="inlineStr">
         <is>
           <t>Hoja robusta para caza. Aplica Sangrado con 3+ éxitos.</t>
         </is>
@@ -898,7 +919,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>No Aplica</t>
+          <t>Cualquiera</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -913,10 +934,15 @@
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
+          <t>No Aplica</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
           <t>Escasa</t>
         </is>
       </c>
-      <c r="R5" s="2" t="inlineStr">
+      <c r="S5" s="2" t="inlineStr">
         <is>
           <t>Mochila resistente para expediciones largas.</t>
         </is>
@@ -980,14 +1006,14 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
+          <t>No Aplica</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
           <t>+1 Defensa</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>No Aplica</t>
-        </is>
-      </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
           <t>No Aplica</t>
@@ -995,10 +1021,15 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
+          <t>No Aplica</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
           <t>Escasa</t>
         </is>
       </c>
-      <c r="R6" s="2" t="inlineStr">
+      <c r="S6" s="2" t="inlineStr">
         <is>
           <t>Chaleco reforzado de cuero curtido. Protección ligera sin sacrificar movilidad.</t>
         </is>
@@ -1072,25 +1103,30 @@
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
+          <t>Qué Subcategoría acepta si es contenedor (ej: 'Flechas'), o 'Cualquiera' si no restringe. 'No Aplica' si no es contenedor.</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
           <t>+1 Resistencia o 'No Aplica'</t>
         </is>
       </c>
-      <c r="O7" s="3" t="inlineStr">
+      <c r="P7" s="3" t="inlineStr">
         <is>
           <t>EST001 a EST011 o 'No Aplica'</t>
         </is>
       </c>
-      <c r="P7" s="3" t="inlineStr">
+      <c r="Q7" s="3" t="inlineStr">
         <is>
           <t>EST001 a EST011 o 'No Aplica'</t>
         </is>
       </c>
-      <c r="Q7" s="3" t="inlineStr">
+      <c r="R7" s="3" t="inlineStr">
         <is>
           <t>Común / Escasa / Rara / Muy Rara / Única</t>
         </is>
       </c>
-      <c r="R7" s="3" t="inlineStr">
+      <c r="S7" s="3" t="inlineStr">
         <is>
           <t>Descripción narrativa del item</t>
         </is>

</xml_diff>